<commit_message>
added redlight to exosome
</commit_message>
<xml_diff>
--- a/spreadsheets/pricing.xlsx
+++ b/spreadsheets/pricing.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="99">
   <si>
     <t>WAX</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Chin</t>
   </si>
   <si>
-    <t>Ears</t>
-  </si>
-  <si>
     <t>Full Arm</t>
   </si>
   <si>
@@ -87,9 +84,6 @@
   </si>
   <si>
     <t>Lower Leg</t>
-  </si>
-  <si>
-    <t>Feet &amp; Toes</t>
   </si>
   <si>
     <t>Bikini</t>
@@ -222,7 +216,7 @@
     <t>*NEW* Exosome+V Renewal Oxygen Facial</t>
   </si>
   <si>
-    <t xml:space="preserve">An advanced post-nano microneedling treatment featuring Intraceuticals’ Exosome+V Serum, infused with vegan biomimetic exosomes, vitamins A, C &amp; E, green tea extract, bioactive peptides, and low-weight hyaluronic acid to support skin communication, renewal, and long-term skin vitality. </t>
+    <t>An advanced post-nano microneedling treatment featuring Intraceuticals’ Exosome+V Serum, infused with vegan biomimetic exosomes, vitamins A, C &amp; E, green tea extract, bioactive peptides, and low-weight hyaluronic acid to support skin communication, renewal, and long-term skin vitality. Finished with LED light therapy to further support skin renewal and recovery.</t>
   </si>
   <si>
     <t>Mona's Glow Facial</t>
@@ -235,20 +229,6 @@
   </si>
   <si>
     <t>A European facial with the addition of Sothys Lactic Acid Peel that resurfaces superficial lines and stimulates cell rejuvenation and brightening. Followed by a manual extraction and Mona's unique signature massage. Topping the treatment with a soothing ampule and Sothys W+ Illuminating Mask to complete this non-irritating acid treatment.</t>
-  </si>
-  <si>
-    <t>Detox Energie</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color indexed="11"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Detox Energie is an intensive detoxifying energizing treatment that gives the skin a burst of energy, helping it defend itself against environmental stress which can accelerate skin aging. Detox Energie is a six step treatment of intense detoxifying, exfoliation, antipollution protection, oxygenation of the skin using Digi-Esthétique Massage rebalancing, and detox using ingredients such as Elderberry, Siberian Ginseng, Peptides, Marshmallow extract, Vitamin C, and Marine complex, leaving the skin energized and radiant!
-</t>
-    </r>
   </si>
   <si>
     <t>Organic Certified Radiance Treatment by Sothys Organics®</t>
@@ -269,6 +249,20 @@
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Detox Energie</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color indexed="11"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">Detox Energie is an intensive detoxifying energizing treatment that gives the skin a burst of energy, helping it defend itself against environmental stress which can accelerate skin aging. Detox Energie is a six step treatment of intense detoxifying, exfoliation, antipollution protection, oxygenation of the skin using Digi-Esthétique Massage rebalancing, and detox using ingredients such as Elderberry, Siberian Ginseng, Peptides, Marshmallow extract, Vitamin C, and Marine complex, leaving the skin energized and radiant!
 </t>
     </r>
   </si>
@@ -1739,7 +1733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="9" width="14.5" style="1" customWidth="1"/>
@@ -1961,10 +1955,10 @@
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="5">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="E13" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -1978,10 +1972,10 @@
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="5">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="E14" s="5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -2012,10 +2006,10 @@
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="5">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E16" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -2029,10 +2023,10 @@
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="5">
-        <v>18</v>
+        <v>95</v>
       </c>
       <c r="E17" s="5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -2046,10 +2040,10 @@
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="5">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="E18" s="5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -2063,7 +2057,7 @@
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="5">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="E19" s="5">
         <v>15</v>
@@ -2097,10 +2091,10 @@
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="5">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="E21" s="5">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -2114,10 +2108,10 @@
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="5">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E22" s="5">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -2131,10 +2125,10 @@
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="5">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E23" s="5">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -2148,10 +2142,10 @@
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="5">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="E24" s="5">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -2165,10 +2159,10 @@
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="5">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="E25" s="5">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -2182,10 +2176,10 @@
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="5">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E26" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -2194,12 +2188,10 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="3"/>
-      <c r="B27" t="s" s="4">
-        <v>30</v>
-      </c>
+      <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="5">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E27" s="5">
         <v>15</v>
@@ -2209,18 +2201,12 @@
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" ht="13.65" customHeight="1">
       <c r="A28" s="3"/>
-      <c r="B28" t="s" s="4">
-        <v>31</v>
-      </c>
+      <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="5">
-        <v>18</v>
-      </c>
-      <c r="E28" s="5">
-        <v>10</v>
-      </c>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
@@ -2230,18 +2216,16 @@
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
-      <c r="D29" s="5">
-        <v>30</v>
-      </c>
-      <c r="E29" s="5">
-        <v>15</v>
-      </c>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-    </row>
-    <row r="30" ht="13.65" customHeight="1">
+      <c r="I29" t="s" s="6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -2250,32 +2234,8 @@
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-      <c r="I31" t="s" s="6">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" t="s" s="6">
-        <v>33</v>
+      <c r="I30" t="s" s="6">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -2299,7 +2259,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" t="s" s="8">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s" s="8">
         <v>1</v>
@@ -2319,7 +2279,7 @@
     </row>
     <row r="2" ht="191.95" customHeight="1">
       <c r="A2" t="s" s="9">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -2330,17 +2290,17 @@
         <v>90</v>
       </c>
       <c r="F2" t="s" s="12">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" t="s" s="9">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
       <c r="D3" t="s" s="9">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E3" s="11">
         <v>90</v>
@@ -2349,7 +2309,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" t="s" s="9">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -2360,12 +2320,12 @@
         <v>90</v>
       </c>
       <c r="F4" t="s" s="14">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" t="s" s="15">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -2376,12 +2336,12 @@
         <v>90</v>
       </c>
       <c r="F5" t="s" s="14">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" t="s" s="6">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -2392,12 +2352,12 @@
         <v>60</v>
       </c>
       <c r="F6" t="s" s="9">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" t="s" s="6">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -2408,44 +2368,44 @@
         <v>60</v>
       </c>
       <c r="F7" t="s" s="9">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" t="s" s="9">
-        <v>47</v>
+      <c r="A8" t="s" s="6">
+        <v>45</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="11">
-        <v>185</v>
+        <v>145</v>
       </c>
       <c r="E8" s="11">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s" s="12">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" t="s" s="6">
-        <v>49</v>
+      <c r="A9" t="s" s="9">
+        <v>47</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="11">
-        <v>145</v>
+        <v>185</v>
       </c>
       <c r="E9" s="11">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s" s="12">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" t="s" s="6">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -2456,12 +2416,12 @@
         <v>60</v>
       </c>
       <c r="F10" t="s" s="9">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" t="s" s="6">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -2472,12 +2432,12 @@
         <v>70</v>
       </c>
       <c r="F11" t="s" s="12">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" t="s" s="6">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -2488,12 +2448,12 @@
         <v>30</v>
       </c>
       <c r="F12" t="s" s="12">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" t="s" s="6">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -2504,12 +2464,12 @@
         <v>70</v>
       </c>
       <c r="F13" t="s" s="12">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" t="s" s="6">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -2520,12 +2480,12 @@
         <v>60</v>
       </c>
       <c r="F14" t="s" s="12">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" t="s" s="6">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -2536,12 +2496,12 @@
         <v>45</v>
       </c>
       <c r="F15" t="s" s="12">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" t="s" s="6">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
@@ -2552,17 +2512,17 @@
         <v>60</v>
       </c>
       <c r="F16" t="s" s="9">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" t="s" s="6">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" t="s" s="9">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E17" s="11">
         <v>60</v>
@@ -2571,7 +2531,7 @@
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" t="s" s="6">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -2604,7 +2564,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s" s="2">
         <v>1</v>
@@ -2619,33 +2579,33 @@
         <v>4</v>
       </c>
       <c r="F1" t="s" s="2">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" ht="332.85" customHeight="1">
       <c r="A2" s="18"/>
       <c r="B2" t="s" s="19">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C2" s="18"/>
       <c r="D2" t="s" s="20">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E2" s="5">
         <v>55</v>
       </c>
       <c r="F2" t="s" s="21">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" ht="78.85" customHeight="1">
       <c r="A3" s="18"/>
       <c r="B3" t="s" s="19">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C3" s="18"/>
       <c r="D3" t="s" s="20">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E3" s="5">
         <v>55</v>
@@ -2655,59 +2615,59 @@
     <row r="4" ht="332.85" customHeight="1">
       <c r="A4" s="18"/>
       <c r="B4" t="s" s="6">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C4" s="18"/>
       <c r="D4" t="s" s="20">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E4" s="5">
         <v>60</v>
       </c>
       <c r="F4" t="s" s="21">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" t="s" s="6">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" t="s" s="20">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E5" s="5">
         <v>55</v>
       </c>
       <c r="F5" t="s" s="6">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" t="s" s="6">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" t="s" s="20">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E6" s="5">
         <v>55</v>
       </c>
       <c r="F6" t="s" s="6">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" t="s" s="6">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" t="s" s="20">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E7" s="5">
         <v>55</v>
@@ -2717,33 +2677,33 @@
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" t="s" s="6">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" t="s" s="20">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E8" s="5">
         <v>55</v>
       </c>
       <c r="F8" t="s" s="6">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" t="s" s="6">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" t="s" s="20">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E9" s="5">
         <v>75</v>
       </c>
       <c r="F9" t="s" s="6">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
@@ -2782,7 +2742,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" t="s" s="2">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B1" t="s" s="2">
         <v>1</v>
@@ -2800,10 +2760,10 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="3"/>
       <c r="B2" t="s" s="6">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s" s="6">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D2" s="5">
         <v>120</v>
@@ -2815,7 +2775,7 @@
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3"/>
       <c r="B3" t="s" s="6">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="5">
@@ -2828,7 +2788,7 @@
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" t="s" s="6">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="5">
@@ -2841,7 +2801,7 @@
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" t="s" s="6">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="5">
@@ -2854,7 +2814,7 @@
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" t="s" s="6">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="5">
@@ -2867,7 +2827,7 @@
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" t="s" s="6">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="5">
@@ -2880,7 +2840,7 @@
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" t="s" s="6">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="5">
@@ -2893,7 +2853,7 @@
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" t="s" s="6">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="5">
@@ -2906,7 +2866,7 @@
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="3"/>
       <c r="B10" t="s" s="6">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="5">

</xml_diff>